<commit_message>
Add PRD cross-reference column to compliance requirements
Flags overlap level (None/Low/Moderate/High) and cites the specific
PRD section or NFR each requirement maps to, so Compliance and
Product can reconcile duplicated items before finalizing.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Msiz5p6hoKmmUHZyLJTkqb
</commit_message>
<xml_diff>
--- a/Visa Compliance Requirements.xlsx
+++ b/Visa Compliance Requirements.xlsx
@@ -50,7 +50,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -71,8 +71,38 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00F8CBAD"/>
+        <bgColor rgb="00F8CBAD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00E2EFDA"/>
         <bgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C9DCF0"/>
+        <bgColor rgb="00C9DCF0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+        <bgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FBD4B4"/>
+        <bgColor rgb="00FBD4B4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+        <bgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
   </fills>
@@ -102,7 +132,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -123,6 +153,21 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -490,14 +535,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="55" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -540,6 +587,16 @@
           <t>Requirement Type</t>
         </is>
       </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>PRD Overlap Level</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>PRD Cross-Reference (Location / Notes)</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="120" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -567,6 +624,16 @@
           <t>Non-Functional</t>
         </is>
       </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>PRD NFR 1.1 (Fraud Detection): "Fraud monitoring system must be active and must identify and flag fraudulent transactions in near real-time" (≥95% detected). Reconcile ownership/wording with Product before finalizing.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="105" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
@@ -589,13 +656,23 @@
           <t>Given that a fraud alert has been generated in Everlink eDetect, When the Fraud Specialist reviews the alert, Then the Fraud Specialist shall disposition the alert (e.g., confirmed fraud, false positive) and document the outcome per the SOP.</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="E6" s="8" t="inlineStr">
         <is>
           <t>Functional</t>
         </is>
       </c>
-    </row>
-    <row r="7" ht="120" customHeight="1">
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>Low-Moderate</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>PRD NFR 1.3 (Fraud Response Actions): "System must support immediate transaction suspension upon detection of fraud" (system SLA, not the investigation/disposition workflow itself) — complementary, not duplicate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="135" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>1.3</t>
@@ -616,9 +693,19 @@
           <t>Given that a cardholder has submitted a fraud dispute, When the Fraud Specialist investigates the dispute, Then the Fraud Specialist shall review transaction activity, customer history, authentication results, and supporting evidence, and reach a documented determination within Visa's required timeframes.</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="E7" s="8" t="inlineStr">
         <is>
           <t>Functional</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>PRD Section 5 (Disputes &amp; Chargebacks): "Support end-to-end dispute lifecycle mgmt including intake, investigation, tracking, resolution, and closure for all dispute types." Reconcile so platform capability and Compliance's investigation obligation aren't documented twice.</t>
         </is>
       </c>
     </row>
@@ -643,9 +730,19 @@
           <t>Given that a transaction is under fraud investigation or review, When the Fraud Specialist accesses Everlink eAuthenticate, Then the Fraud Specialist shall be able to view the authentication results and transaction details needed to support the investigation and decisioning.</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
+      <c r="E8" s="8" t="inlineStr">
         <is>
           <t>Functional</t>
+        </is>
+      </c>
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>No mention of eAuthenticate anywhere in the PRD. Net new.</t>
         </is>
       </c>
     </row>
@@ -670,13 +767,23 @@
           <t>Given that a cardholder's dispute activity is tracked on an ongoing basis, When a cardholder reaches 5 or more disputes within a rolling 12-month period, Then a formal review of the cardholder's account and dispute pattern shall be triggered and documented.</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr">
+      <c r="E9" s="8" t="inlineStr">
         <is>
           <t>Functional</t>
         </is>
       </c>
-    </row>
-    <row r="10" ht="120" customHeight="1">
+      <c r="F9" s="10" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>No mention of a 5+ disputes/12-month first-party fraud threshold anywhere in the PRD. Net new.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="135" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>1.6</t>
@@ -702,8 +809,18 @@
           <t>Non-Functional</t>
         </is>
       </c>
-    </row>
-    <row r="11" ht="105" customHeight="1">
+      <c r="F10" s="11" t="inlineStr">
+        <is>
+          <t>Moderate-High</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>PRD NFR 1.2/1.4 (centralized fraud data repository; fraud data provided to Everlink on ongoing basis) and Fraud Loss Rate / Dispute Rate metrics in the Data, Metrics &amp; Telemetry section. Existing items are system/data-feed focused; ours adds the governance reporting deliverable — reconcile.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="120" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>1.7</t>
@@ -727,6 +844,16 @@
       <c r="E11" s="6" t="inlineStr">
         <is>
           <t>Non-Functional</t>
+        </is>
+      </c>
+      <c r="F11" s="10" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>No mention of eAuthenticate failure analysis anywhere in the PRD. Net new.</t>
         </is>
       </c>
     </row>
@@ -751,16 +878,26 @@
           <t>Given that a cardholder dispute has been confirmed as fraud, When the Fraud Specialist prepares the dispute case for submission, Then the case shall be packaged with all required documentation and provided to Everlink for submission to VROL within Visa's mandated timeframe.</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr">
+      <c r="E12" s="8" t="inlineStr">
         <is>
           <t>Functional</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>PRD NFR 1.6 ("System must support reporting of fraud data to Visa via VROL") and Section 5 ("Dispute mgmt platform integrates with VROL for chargeback submission, fraud reporting, evidence exchange"). Reconcile system-capability language with this operational preparation step.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -772,14 +909,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="55" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -822,6 +961,16 @@
           <t>Requirement Type</t>
         </is>
       </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>PRD Overlap Level</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>PRD Cross-Reference (Location / Notes)</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="120" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -844,9 +993,19 @@
           <t>Given that Visa Debit transaction activity is monitored by the AML monitoring system (Navaera), When an alert is generated for potentially suspicious activity, Then the AML Specialist shall investigate and disposition the alert (e.g., cleared, escalated, STR filed) and document the outcome.</t>
         </is>
       </c>
-      <c r="E5" s="7" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr">
         <is>
           <t>Functional</t>
+        </is>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>PRD NFR 1.10: "All applicable AML and KYC compliance processes must be supported" — a generic one-line placeholder with no operational detail. Ours substantially fleshes it out rather than duplicating it.</t>
         </is>
       </c>
     </row>
@@ -876,8 +1035,18 @@
           <t>Non-Functional</t>
         </is>
       </c>
-    </row>
-    <row r="7" ht="120" customHeight="1">
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>"OFAC" and "sanctions" do not appear anywhere in the PRD. Net new.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="135" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>2.3</t>
@@ -898,9 +1067,19 @@
           <t>Given that Visa Debit transaction activity meets or is suspected to meet FINTRAC reporting criteria, When the AML Specialist assesses the transaction, Then the AML Specialist shall determine whether an STR, EFT, and/or LCT report is required and document the assessment.</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="E7" s="8" t="inlineStr">
         <is>
           <t>Functional</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>PRD NFR 1.11 ("All applicable reporting requirements (eg: FINTRAC) must be supported") and Section 7 Data Reporting: "Ability to support Fintrac Reporting... It is still TBD whether this will be used" (marked WIP). This isn't duplication so much as resolving an item Beem already flagged as open.</t>
         </is>
       </c>
     </row>
@@ -925,9 +1104,19 @@
           <t>Given that a regulatory reporting obligation (e.g., STR, EFT, LCT) has been identified for Visa Debit activity, When the AML Specialist prepares the report, Then the report shall be submitted to FINTRAC within the applicable regulatory timeframe and retained per record-keeping requirements.</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
+      <c r="E8" s="8" t="inlineStr">
         <is>
           <t>Functional</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Same FINTRAC placeholder as 2.3 — PRD NFR 1.11 and Section 7's WIP "Ability to support Fintrac Reporting" item. Reconcile together with 2.3.</t>
         </is>
       </c>
     </row>
@@ -957,8 +1146,18 @@
           <t>Non-Functional</t>
         </is>
       </c>
-    </row>
-    <row r="10" ht="105" customHeight="1">
+      <c r="F9" s="12" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>Only the generic NFR 1.10 ("AML and KYC compliance processes must be supported") touches this indirectly. No dedicated AML management reporting item exists in the PRD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="120" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>2.6</t>
@@ -982,13 +1181,23 @@
       <c r="E10" s="6" t="inlineStr">
         <is>
           <t>Non-Functional</t>
+        </is>
+      </c>
+      <c r="F10" s="12" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>Adjacent to a Maintenance &amp; Scale NFR on configurable "fraud thresholds" via admin settings — but that item is fraud-specific, not AML rule tuning. Largely net new.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1000,14 +1209,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="55" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -1050,6 +1261,16 @@
           <t>Requirement Type</t>
         </is>
       </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>PRD Overlap Level</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>PRD Cross-Reference (Location / Notes)</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="135" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -1072,13 +1293,23 @@
           <t>Given that a net new TPA is being onboarded to support the Visa Debit program, When Compliance performs the compliance due diligence review, Then the TPA's compliance-related documentation and controls shall be reviewed and a compliance due diligence determination shall be documented prior to the TPA being onboarded.</t>
         </is>
       </c>
-      <c r="E5" s="7" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr">
         <is>
           <t>Functional</t>
         </is>
       </c>
-    </row>
-    <row r="6" ht="135" customHeight="1">
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>The PRD contains no TPA/TPRM content anywhere ("third party," "TPA," "vendor," and "TPRM" do not appear). This entire section is net new.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="150" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>3.2</t>
@@ -1099,13 +1330,23 @@
           <t>Given that a TPA is registered, a TPA contract change occurs, or Visa/the BIN Sponsor requests quarterly TPA reporting, When Compliance prepares the applicable TPA report or notification, Then the report/notification shall be submitted to Visa and/or the BIN Sponsor within the applicable timeframe (e.g., within 5 business days for contract changes).</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="E6" s="8" t="inlineStr">
         <is>
           <t>Functional</t>
         </is>
       </c>
-    </row>
-    <row r="7" ht="105" customHeight="1">
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>No TPA reporting content in the PRD. Net new.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="120" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>3.3</t>
@@ -1126,16 +1367,26 @@
           <t>Given that a net new TPA agreement is being drafted or finalized, When Compliance reviews the agreement, Then Compliance shall confirm the agreement includes the Visa-required contractual provisions and shall document any gaps or required amendments prior to execution.</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="E7" s="8" t="inlineStr">
         <is>
           <t>Functional</t>
+        </is>
+      </c>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>No TPA agreement/contract review content in the PRD. Net new.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Address manager feedback: strip vendor names, add system-level functional requirements
- Removed all vendor/product names (Navaera, Everlink, eDetect, eAuthenticate)
  in favor of generic system references
- Reclassified all specialist-actor requirements (Fraud/AML Specialist) as
  Non-Functional
- Added new Functional requirements with system actors (Fraud/AML Monitoring
  System) covering: business rule management, sanctions screening, masked
  data export via API, interactive dashboards (+ NF availability pair),
  automated held-transaction alerts, and analytics/performance reporting

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Msiz5p6hoKmmUHZyLJTkqb
</commit_message>
<xml_diff>
--- a/Visa Compliance Requirements.xlsx
+++ b/Visa Compliance Requirements.xlsx
@@ -77,12 +77,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
-        <bgColor rgb="00E2EFDA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00C9DCF0"/>
         <bgColor rgb="00C9DCF0"/>
       </patternFill>
@@ -97,6 +91,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FBD4B4"/>
         <bgColor rgb="00FBD4B4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+        <bgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
@@ -535,7 +535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -616,7 +616,7 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Given that Visa Debit transaction activity is occurring across the member base, When the fraud monitoring solution (Everlink eDetect) evaluates transactions against fraud rules, Then any transaction meeting fraud criteria shall generate an alert for Fraud Specialist review.</t>
+          <t>Given that Visa Debit transaction activity is occurring across the member base, When the fraud monitoring system evaluates transactions against fraud rules, Then any transaction meeting fraud criteria shall generate an alert for Fraud Specialist review.</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
@@ -635,7 +635,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="105" customHeight="1">
+    <row r="6" ht="120" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>1.2</t>
@@ -643,25 +643,25 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>As a Fraud Specialist, I want to investigate and disposition debit card fraud events flagged in Everlink eDetect, So that confirmed fraud is actioned and false positives are cleared in accordance with established SOPs</t>
+          <t>As a Fraud Specialist, I want to investigate and disposition debit card fraud events flagged in the fraud monitoring system, So that confirmed fraud is actioned and false positives are cleared in accordance with established SOPs</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Beem shall investigate and disposition all debit card fraud events flagged in Everlink eDetect in accordance with established SOPs.</t>
+          <t>Beem shall investigate and disposition all debit card fraud events flagged in the fraud monitoring system in accordance with established SOPs.</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Given that a fraud alert has been generated in Everlink eDetect, When the Fraud Specialist reviews the alert, Then the Fraud Specialist shall disposition the alert (e.g., confirmed fraud, false positive) and document the outcome per the SOP.</t>
-        </is>
-      </c>
-      <c r="E6" s="8" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="F6" s="9" t="inlineStr">
+          <t>Given that a fraud alert has been generated in the fraud monitoring system, When the Fraud Specialist reviews the alert, Then the Fraud Specialist shall disposition the alert (e.g., confirmed fraud, false positive) and document the outcome per the SOP.</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Non-Functional</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
         <is>
           <t>Low-Moderate</t>
         </is>
@@ -693,9 +693,9 @@
           <t>Given that a cardholder has submitted a fraud dispute, When the Fraud Specialist investigates the dispute, Then the Fraud Specialist shall review transaction activity, customer history, authentication results, and supporting evidence, and reach a documented determination within Visa's required timeframes.</t>
         </is>
       </c>
-      <c r="E7" s="8" t="inlineStr">
-        <is>
-          <t>Functional</t>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>Non-Functional</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
@@ -717,32 +717,32 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>As a Fraud Specialist, I want to review transaction activity in Everlink eAuthenticate, So that I can support fraud investigations, authentication review, and transaction-level decisioning</t>
+          <t>As a Fraud Specialist, I want to review transaction activity in the authentication system, So that I can support fraud investigations, authentication review, and transaction-level decisioning</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Beem shall use Everlink eAuthenticate to review transaction-level authentication activity in support of fraud investigations and decisioning.</t>
+          <t>Beem shall use the authentication system to review transaction-level authentication activity in support of fraud investigations and decisioning.</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Given that a transaction is under fraud investigation or review, When the Fraud Specialist accesses Everlink eAuthenticate, Then the Fraud Specialist shall be able to view the authentication results and transaction details needed to support the investigation and decisioning.</t>
-        </is>
-      </c>
-      <c r="E8" s="8" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="F8" s="10" t="inlineStr">
+          <t>Given that a transaction is under fraud investigation or review, When the Fraud Specialist accesses the authentication system, Then the Fraud Specialist shall be able to view the authentication results and transaction details needed to support the investigation and decisioning.</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>Non-Functional</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>No mention of eAuthenticate anywhere in the PRD. Net new.</t>
+          <t>No mention of an authentication review system anywhere in the PRD. Net new.</t>
         </is>
       </c>
     </row>
@@ -767,12 +767,12 @@
           <t>Given that a cardholder's dispute activity is tracked on an ongoing basis, When a cardholder reaches 5 or more disputes within a rolling 12-month period, Then a formal review of the cardholder's account and dispute pattern shall be triggered and documented.</t>
         </is>
       </c>
-      <c r="E9" s="8" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="F9" s="10" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>Non-Functional</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
         <is>
           <t>None</t>
         </is>
@@ -791,12 +791,12 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>As a Fraud Specialist, I want to prepare fraud loss reporting and governance reporting in coordination with Everlink, So that fraud volumes, loss trends, recoveries, aging, and key risk indicators are visible to management and governance stakeholders</t>
+          <t>As a Fraud Specialist, I want to prepare fraud loss reporting and governance reporting in coordination with the processor, So that fraud volumes, loss trends, recoveries, aging, and key risk indicators are visible to management and governance stakeholders</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Beem shall prepare fraud loss and governance reporting, in coordination with Everlink, on a regular basis, including fraud volumes, loss trends, recoveries, aging, and key risk indicators.</t>
+          <t>Beem shall prepare fraud loss and governance reporting, in coordination with the processor, on a regular basis, including fraud volumes, loss trends, recoveries, aging, and key risk indicators.</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
@@ -809,14 +809,14 @@
           <t>Non-Functional</t>
         </is>
       </c>
-      <c r="F10" s="11" t="inlineStr">
+      <c r="F10" s="10" t="inlineStr">
         <is>
           <t>Moderate-High</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>PRD NFR 1.2/1.4 (centralized fraud data repository; fraud data provided to Everlink on ongoing basis) and Fraud Loss Rate / Dispute Rate metrics in the Data, Metrics &amp; Telemetry section. Existing items are system/data-feed focused; ours adds the governance reporting deliverable — reconcile.</t>
+          <t>PRD NFR 1.2/1.4 (centralized fraud data repository; fraud data provided to the processor on ongoing basis) and Fraud Loss Rate / Dispute Rate metrics in the Data, Metrics &amp; Telemetry section. Existing items are system/data-feed focused; ours adds the governance reporting deliverable — reconcile.</t>
         </is>
       </c>
     </row>
@@ -828,17 +828,17 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>As a Fraud Specialist, I want to analyze eAuthenticate failures on an ongoing basis, So that I can identify patterns, root causes, and potential fraud-rule tuning opportunities</t>
+          <t>As a Fraud Specialist, I want to analyze authentication failures on an ongoing basis, So that I can identify patterns, root causes, and potential fraud-rule tuning opportunities</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Beem shall analyze eAuthenticate failures on an ongoing basis to identify patterns, root causes, and opportunities for fraud-rule tuning.</t>
+          <t>Beem shall analyze authentication failures on an ongoing basis to identify patterns, root causes, and opportunities for fraud-rule tuning.</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Given that eAuthenticate failure data is available on an ongoing basis, When the Fraud Specialist conducts the periodic failure analysis, Then patterns and root causes shall be identified and documented, and any recommended fraud-rule tuning shall be raised for review.</t>
+          <t>Given that authentication failure data is available on an ongoing basis, When the Fraud Specialist conducts the periodic failure analysis, Then patterns and root causes shall be identified and documented, and any recommended fraud-rule tuning shall be raised for review.</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
@@ -846,14 +846,14 @@
           <t>Non-Functional</t>
         </is>
       </c>
-      <c r="F11" s="10" t="inlineStr">
+      <c r="F11" s="9" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>No mention of eAuthenticate failure analysis anywhere in the PRD. Net new.</t>
+          <t>No mention of authentication failure analysis anywhere in the PRD. Net new.</t>
         </is>
       </c>
     </row>
@@ -865,32 +865,217 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>As a Fraud Specialist, I want to prepare fraudulent disputes for Everlink's submission to Visa VROL, So that fraud disputes are processed through VROL within Visa's required timeframes</t>
+          <t>As a Fraud Specialist, I want to prepare fraudulent disputes for submission to Visa VROL, So that fraud disputes are processed through VROL within Visa's required timeframes</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Beem shall prepare all confirmed fraudulent disputes for submission by Everlink to Visa Resolve Online (VROL) within Visa's required timeframes.</t>
+          <t>Beem shall prepare all confirmed fraudulent disputes for submission to Visa Resolve Online (VROL) within Visa's required timeframes.</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Given that a cardholder dispute has been confirmed as fraud, When the Fraud Specialist prepares the dispute case for submission, Then the case shall be packaged with all required documentation and provided to Everlink for submission to VROL within Visa's mandated timeframe.</t>
-        </is>
-      </c>
-      <c r="E12" s="8" t="inlineStr">
+          <t>Given that a cardholder dispute has been confirmed as fraud, When the Fraud Specialist prepares the dispute case for submission, Then the case shall be packaged with all required documentation and provided for submission to VROL within Visa's mandated timeframe.</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>Non-Functional</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>PRD NFR 1.6 ("System must support reporting of fraud data to Visa via VROL") and Section 5 ("Dispute mgmt platform integrates with VROL for chargeback submission, fraud reporting, evidence exchange"). Reconcile system-capability language with this operational preparation step.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="150" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>As a Fraud Monitoring System, I want to support the deployment, creation, modification, and deactivation of business rules in the production environment, across varying rule lengths, variables, rule syntax, and logic complexities, So that Fraud Specialists can configure and maintain effective fraud detection logic without requiring a code deployment</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>The fraud monitoring system shall support the deployment, creation, modification, and deactivation of business rules in the production environment, supporting varying rule lengths, variables, rule syntax, and logic complexities.</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Given that a Fraud Specialist has defined a new or modified business rule, When the rule is deployed, created, modified, or deactivated in the production environment, Then the system shall apply the change without requiring a code deployment or application restart, regardless of the rule's length, variables, syntax, or logic complexity.</t>
+        </is>
+      </c>
+      <c r="E13" s="11" t="inlineStr">
         <is>
           <t>Functional</t>
         </is>
       </c>
-      <c r="F12" s="7" t="inlineStr">
+      <c r="F13" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>PRD NFR 1.6 ("System must support reporting of fraud data to Visa via VROL") and Section 5 ("Dispute mgmt platform integrates with VROL for chargeback submission, fraud reporting, evidence exchange"). Reconcile system-capability language with this operational preparation step.</t>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>PRD NFR (Maintenance &amp; Scale): "Configuration-driven business rules allow admin functions (such as card limits, transaction controls, fraud thresholds, alerts) to be configurable via administrative settings without requiring code deployment / application restart." Reconcile wording/ownership.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="105" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>1.10</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>As a Fraud Monitoring System, I want to provide interactive dashboards displaying solution health, transaction volumes, and alert activity, So that Fraud Specialists can monitor the fraud program's operational status in real time</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>The fraud monitoring system shall provide interactive dashboards displaying solution health, transaction volumes, and alert activity for ongoing monitoring by the Fraud Specialist team.</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Given that the fraud monitoring system is in production, When a Fraud Specialist accesses the dashboard, Then the dashboard shall display current solution health status, transaction volumes, and alert activity, filterable by date range and status.</t>
+        </is>
+      </c>
+      <c r="E14" s="11" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>No mention of fraud monitoring dashboards anywhere in the PRD. Net new.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="120" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>1.11</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>As a Fraud Specialist, I want the fraud monitoring dashboards to be reliably available and performant, So that I can monitor solution health, volumes, and alerts without delay or downtime</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>The fraud monitoring dashboards shall be available and performant, refreshing dashboard data within a defined interval and meeting Beem's system availability standards.</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Given that the fraud monitoring dashboard is in use, When dashboard data is refreshed, Then updated volumes, alerts, and health status shall be reflected within the defined refresh interval, and the dashboard shall be available in accordance with Beem's defined system availability SLA.</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>Non-Functional</t>
+        </is>
+      </c>
+      <c r="F15" s="12" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>Adjacent to the general Availability &amp; Performance NFRs (e.g., ≥99.99% system availability), but those are not dashboard-specific. Largely net new.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="105" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>1.12</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>As a Fraud Monitoring System, I want to automatically generate alerts for held transactions and send them to downstream systems in real time, So that held transactions are actioned promptly by the appropriate team or system</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>The fraud monitoring system shall automatically generate an alert for each held transaction and transmit the alert to downstream systems in real time.</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Given that a transaction is held by the fraud monitoring system, When the hold is applied, Then an alert shall be automatically generated and transmitted to the applicable downstream system(s) in real time.</t>
+        </is>
+      </c>
+      <c r="E16" s="11" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>Low-Moderate</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>Adjacent to PRD NFR 1.3 (Fraud Response Actions): "System must support immediate transaction suspension upon detection of fraud... ≤5 seconds" — that NFR covers the suspension action itself, not automated downstream alert generation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="135" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>1.13</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>As a Fraud Monitoring System, I want to allow Fraud Specialists to view, create, and customize analytics and performance reports, So that the team can track and monitor fraud program performance and trends</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>The fraud monitoring system shall allow Fraud Specialists to view, create, and customize analytics and performance reports to track and monitor fraud program performance and trends.</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Given that a Fraud Specialist requires a report to track or monitor fraud program performance, When the Fraud Specialist creates or customizes an analytics or performance report within the fraud monitoring system, Then the report shall be generated and made available for view, export, and ongoing use.</t>
+        </is>
+      </c>
+      <c r="E17" s="11" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="F17" s="12" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>The PRD's Data, Metrics &amp; Telemetry section defines specific metrics (Fraud Loss Rate, Dispute Rate) but does not describe a system capability for Fraud Specialists to create/customize their own reports. Largely net new.</t>
         </is>
       </c>
     </row>
@@ -909,7 +1094,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -990,12 +1175,12 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Given that Visa Debit transaction activity is monitored by the AML monitoring system (Navaera), When an alert is generated for potentially suspicious activity, Then the AML Specialist shall investigate and disposition the alert (e.g., cleared, escalated, STR filed) and document the outcome.</t>
-        </is>
-      </c>
-      <c r="E5" s="8" t="inlineStr">
-        <is>
-          <t>Functional</t>
+          <t>Given that Visa Debit transaction activity is monitored by the AML monitoring system, When an alert is generated for potentially suspicious activity, Then the AML Specialist shall investigate and disposition the alert (e.g., cleared, escalated, STR filed) and document the outcome.</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Non-Functional</t>
         </is>
       </c>
       <c r="F5" s="12" t="inlineStr">
@@ -1022,12 +1207,12 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Beem shall screen all Visa Debit cardholders against OFAC SDN and other applicable sanctions lists at onboarding and on an ongoing basis via Navaera.</t>
+          <t>Beem shall screen all Visa Debit cardholders against OFAC SDN and other applicable sanctions lists at onboarding and on an ongoing basis.</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Given that a cardholder is onboarded or an ongoing sanctions screening cycle occurs, When the cardholder's details are screened against OFAC SDN and other applicable sanctions lists via Navaera, Then any potential match shall be flagged for AML Specialist review and disposition prior to further account activity, where required.</t>
+          <t>Given that a cardholder is onboarded or an ongoing sanctions screening cycle occurs, When the cardholder's details are screened against OFAC SDN and other applicable sanctions lists, Then any potential match shall be flagged for AML Specialist review and disposition prior to further account activity, where required.</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -1035,7 +1220,7 @@
           <t>Non-Functional</t>
         </is>
       </c>
-      <c r="F6" s="10" t="inlineStr">
+      <c r="F6" s="9" t="inlineStr">
         <is>
           <t>None</t>
         </is>
@@ -1067,9 +1252,9 @@
           <t>Given that Visa Debit transaction activity meets or is suspected to meet FINTRAC reporting criteria, When the AML Specialist assesses the transaction, Then the AML Specialist shall determine whether an STR, EFT, and/or LCT report is required and document the assessment.</t>
         </is>
       </c>
-      <c r="E7" s="8" t="inlineStr">
-        <is>
-          <t>Functional</t>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>Non-Functional</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
@@ -1104,9 +1289,9 @@
           <t>Given that a regulatory reporting obligation (e.g., STR, EFT, LCT) has been identified for Visa Debit activity, When the AML Specialist prepares the report, Then the report shall be submitted to FINTRAC within the applicable regulatory timeframe and retained per record-keeping requirements.</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
-        <is>
-          <t>Functional</t>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>Non-Functional</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
@@ -1175,7 +1360,7 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Given that Visa Debit AML monitoring rules are in production, When the AML Specialist conducts periodic rule review and tuning, Then rule changes shall be assessed, tested, and documented, and approved changes shall be implemented in the monitoring system (Navaera).</t>
+          <t>Given that Visa Debit AML monitoring rules are in production, When the AML Specialist conducts periodic rule review and tuning, Then rule changes shall be assessed, tested, and documented, and approved changes shall be implemented in the AML monitoring system.</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
@@ -1191,6 +1376,228 @@
       <c r="G10" s="5" t="inlineStr">
         <is>
           <t>Adjacent to a Maintenance &amp; Scale NFR on configurable "fraud thresholds" via admin settings — but that item is fraud-specific, not AML rule tuning. Largely net new.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="150" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>2.7</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>As an AML Monitoring System, I want to support the deployment, creation, modification, and deactivation of business rules in the production environment, across varying rule lengths, variables, rule syntax, and logic complexities, So that AML Specialists can configure and maintain effective AML detection logic without requiring a code deployment</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>The AML monitoring system shall support the deployment, creation, modification, and deactivation of business rules in the production environment, supporting varying rule lengths, variables, rule syntax, and logic complexities.</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Given that an AML Specialist has defined a new or modified business rule, When the rule is deployed, created, modified, or deactivated in the production environment, Then the system shall apply the change without requiring a code deployment or application restart, regardless of the rule's length, variables, syntax, or logic complexity.</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="F11" s="12" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>Adjacent to the PRD's Maintenance &amp; Scale NFR on configurable "fraud thresholds" via admin settings — that item is fraud-specific, not AML rule configuration. Largely net new.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="150" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>2.8</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>As an AML Monitoring System, I want to screen cardholders against the OFAC Specially Designated Nationals and Blocked Persons List (SDN List) and other applicable sanctions lists at onboarding/issuance and on an ongoing basis, So that true matches are actioned immediately to prevent sanctioned individuals from transacting</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>The AML monitoring system shall screen all Visa Debit cardholders against the OFAC Specially Designated Nationals and Blocked Persons List (SDN List) and other applicable sanctions lists at onboarding/card issuance and on an ongoing basis; upon a true match, the system shall disable cardholder access, notify Visa, and report remediation.</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Given that a cardholder is onboarded, issued a Visa Debit card, or included in an ongoing sanctions screening cycle, When the cardholder is screened against the OFAC SDN List and other applicable sanctions lists, Then any true match shall result in the cardholder's access being disabled, Visa being notified, and remediation being reported.</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>Functional (system) counterpart to 2.2. "OFAC"/"sanctions" do not appear anywhere in the PRD. Net new.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="135" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>2.9</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>As an AML Monitoring System, I want to receive Visa Debit card data via an export mechanism such as an API, with sensitive data masked, So that the AML monitoring solution can perform screening, transaction monitoring, and case management on Visa Debit activity</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Beem's systems shall export masked Visa Debit card data (e.g., via API) to make Visa Debit transaction and cardholder data available to the AML monitoring system.</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Given that Visa Debit transaction or cardholder data needs to be made available to the AML monitoring system, When the data export mechanism (e.g., API) runs, Then the data shall be delivered to the AML monitoring system with sensitive data elements masked in accordance with data protection requirements.</t>
+        </is>
+      </c>
+      <c r="E13" s="11" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="F13" s="12" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>Adjacent to general PRD NFRs on data masking and cardholder data protection (Section 2, Security &amp; Data Protection), but none address exporting data specifically to an AML monitoring solution. Largely net new.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="105" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>2.10</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>As an AML Monitoring System, I want to provide interactive dashboards displaying solution health, alert volumes, and case status, So that AML Specialists can monitor the AML program's operational status in real time</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>The AML monitoring system shall provide interactive dashboards displaying solution health, alert volumes, and case status for ongoing monitoring by the AML Specialist team.</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Given that the AML monitoring system is in production, When an AML Specialist accesses the dashboard, Then the dashboard shall display current solution health status, alert volumes, and case status, filterable by date range and status.</t>
+        </is>
+      </c>
+      <c r="E14" s="11" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>No mention of AML monitoring dashboards anywhere in the PRD. Net new.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="120" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>2.11</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>As an AML Specialist, I want the AML monitoring dashboards to be reliably available and performant, So that I can monitor solution health, volumes, and alerts without delay or downtime</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>The AML monitoring dashboards shall be available and performant, refreshing dashboard data within a defined interval and meeting Beem's system availability standards.</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Given that the AML monitoring dashboard is in use, When dashboard data is refreshed, Then updated volumes, alerts, and health status shall be reflected within the defined refresh interval, and the dashboard shall be available in accordance with Beem's defined system availability SLA.</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>Non-Functional</t>
+        </is>
+      </c>
+      <c r="F15" s="12" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>Adjacent to the general Availability &amp; Performance NFRs (e.g., ≥99.99% system availability), but those are not dashboard-specific. Largely net new.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="135" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>2.12</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>As an AML Monitoring System, I want to allow AML Specialists to view, create, and customize analytics and performance reports, So that the team can track and monitor AML program performance and trends</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>The AML monitoring system shall allow AML Specialists to view, create, and customize analytics and performance reports to track and monitor AML program performance and trends.</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Given that an AML Specialist requires a report to track or monitor AML program performance, When the AML Specialist creates or customizes an analytics or performance report within the AML monitoring system, Then the report shall be generated and made available for view, export, and ongoing use.</t>
+        </is>
+      </c>
+      <c r="E16" s="11" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>No mention of AML analytics/performance reporting capability anywhere in the PRD. Net new.</t>
         </is>
       </c>
     </row>
@@ -1293,12 +1700,12 @@
           <t>Given that a net new TPA is being onboarded to support the Visa Debit program, When Compliance performs the compliance due diligence review, Then the TPA's compliance-related documentation and controls shall be reviewed and a compliance due diligence determination shall be documented prior to the TPA being onboarded.</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="E5" s="11" t="inlineStr">
         <is>
           <t>Functional</t>
         </is>
       </c>
-      <c r="F5" s="10" t="inlineStr">
+      <c r="F5" s="9" t="inlineStr">
         <is>
           <t>None</t>
         </is>
@@ -1330,12 +1737,12 @@
           <t>Given that a TPA is registered, a TPA contract change occurs, or Visa/the BIN Sponsor requests quarterly TPA reporting, When Compliance prepares the applicable TPA report or notification, Then the report/notification shall be submitted to Visa and/or the BIN Sponsor within the applicable timeframe (e.g., within 5 business days for contract changes).</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="E6" s="11" t="inlineStr">
         <is>
           <t>Functional</t>
         </is>
       </c>
-      <c r="F6" s="10" t="inlineStr">
+      <c r="F6" s="9" t="inlineStr">
         <is>
           <t>None</t>
         </is>
@@ -1367,12 +1774,12 @@
           <t>Given that a net new TPA agreement is being drafted or finalized, When Compliance reviews the agreement, Then Compliance shall confirm the agreement includes the Visa-required contractual provisions and shall document any gaps or required amendments prior to execution.</t>
         </is>
       </c>
-      <c r="E7" s="8" t="inlineStr">
+      <c r="E7" s="11" t="inlineStr">
         <is>
           <t>Functional</t>
         </is>
       </c>
-      <c r="F7" s="10" t="inlineStr">
+      <c r="F7" s="9" t="inlineStr">
         <is>
           <t>None</t>
         </is>

</xml_diff>

<commit_message>
Bold clause labels and add line breaks in user story / acceptance criteria cells
Bolds "As a/an", "I want", "So that" in User Story and "Given that",
"When", "Then" in Acceptance Criteria, with each clause starting on its
own indented line for readability.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Msiz5p6hoKmmUHZyLJTkqb
</commit_message>
<xml_diff>
--- a/Visa Compliance Requirements.xlsx
+++ b/Visa Compliance Requirements.xlsx
@@ -598,7 +598,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="120" customHeight="1">
+    <row r="5" ht="105" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>1.1</t>
@@ -606,7 +606,47 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>As a Fraud Specialist, I want to monitor Visa Debit transaction activity on an ongoing basis, So that I can identify potential fraud events before they escalate</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>As a</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> Fraud Specialist, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>I want</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> to monitor Visa Debit transaction activity on an ongoing basis, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>So that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> I can identify potential fraud events before they escalate</t>
+          </r>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -616,7 +656,47 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Given that Visa Debit transaction activity is occurring across the member base, When the fraud monitoring system evaluates transactions against fraud rules, Then any transaction meeting fraud criteria shall generate an alert for Fraud Specialist review.</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Given that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> Visa Debit transaction activity is occurring across the member base, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>When</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> the fraud monitoring system evaluates transactions against fraud rules, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Then</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> any transaction meeting fraud criteria shall generate an alert for Fraud Specialist review.</t>
+          </r>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
@@ -643,7 +723,47 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>As a Fraud Specialist, I want to investigate and disposition debit card fraud events flagged in the fraud monitoring system, So that confirmed fraud is actioned and false positives are cleared in accordance with established SOPs</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>As a</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> Fraud Specialist, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>I want</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> to investigate and disposition debit card fraud events flagged in the fraud monitoring system, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>So that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> confirmed fraud is actioned and false positives are cleared in accordance with established SOPs</t>
+          </r>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -653,7 +773,47 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Given that a fraud alert has been generated in the fraud monitoring system, When the Fraud Specialist reviews the alert, Then the Fraud Specialist shall disposition the alert (e.g., confirmed fraud, false positive) and document the outcome per the SOP.</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Given that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> a fraud alert has been generated in the fraud monitoring system, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>When</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> the Fraud Specialist reviews the alert, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Then</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> the Fraud Specialist shall disposition the alert (e.g., confirmed fraud, false positive) and document the outcome per the SOP.</t>
+          </r>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -680,7 +840,47 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>As a Fraud Specialist, I want to investigate fraudulent cardholder disputes by reviewing transaction activity, customer history, authentication results, and supporting evidence, So that I can accurately determine whether a dispute is valid fraud</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>As a</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> Fraud Specialist, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>I want</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> to investigate fraudulent cardholder disputes by reviewing transaction activity, customer history, authentication results, and supporting evidence, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>So that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> I can accurately determine whether a dispute is valid fraud</t>
+          </r>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -690,7 +890,47 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Given that a cardholder has submitted a fraud dispute, When the Fraud Specialist investigates the dispute, Then the Fraud Specialist shall review transaction activity, customer history, authentication results, and supporting evidence, and reach a documented determination within Visa's required timeframes.</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Given that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> a cardholder has submitted a fraud dispute, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>When</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> the Fraud Specialist investigates the dispute, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Then</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> the Fraud Specialist shall review transaction activity, customer history, authentication results, and supporting evidence, and reach a documented determination within Visa's required timeframes.</t>
+          </r>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
@@ -717,7 +957,47 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>As a Fraud Specialist, I want to review transaction activity in the authentication system, So that I can support fraud investigations, authentication review, and transaction-level decisioning</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>As a</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> Fraud Specialist, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>I want</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> to review transaction activity in the authentication system, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>So that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> I can support fraud investigations, authentication review, and transaction-level decisioning</t>
+          </r>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -727,7 +1007,47 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Given that a transaction is under fraud investigation or review, When the Fraud Specialist accesses the authentication system, Then the Fraud Specialist shall be able to view the authentication results and transaction details needed to support the investigation and decisioning.</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Given that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> a transaction is under fraud investigation or review, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>When</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> the Fraud Specialist accesses the authentication system, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Then</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> the Fraud Specialist shall be able to view the authentication results and transaction details needed to support the investigation and decisioning.</t>
+          </r>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
@@ -746,7 +1066,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="120" customHeight="1">
+    <row r="9" ht="135" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
           <t>1.5</t>
@@ -754,7 +1074,47 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>As a Fraud Specialist, I want to monitor and assess cardholders with recurring or excessive dispute activity, So that I can identify potential first-party fraud and comply with Visa's requirement to formally review cardholders with 5 or more disputes in a 12-month period</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>As a</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> Fraud Specialist, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>I want</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> to monitor and assess cardholders with recurring or excessive dispute activity, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>So that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> I can identify potential first-party fraud and comply with Visa's requirement to formally review cardholders with 5 or more disputes in a 12-month period</t>
+          </r>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
@@ -764,7 +1124,47 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Given that a cardholder's dispute activity is tracked on an ongoing basis, When a cardholder reaches 5 or more disputes within a rolling 12-month period, Then a formal review of the cardholder's account and dispute pattern shall be triggered and documented.</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Given that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> a cardholder's dispute activity is tracked on an ongoing basis, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>When</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> a cardholder reaches 5 or more disputes within a rolling 12-month period, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Then</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> a formal review of the cardholder's account and dispute pattern shall be triggered and documented.</t>
+          </r>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
@@ -783,7 +1183,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="135" customHeight="1">
+    <row r="10" ht="120" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>1.6</t>
@@ -791,7 +1191,47 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>As a Fraud Specialist, I want to prepare fraud loss reporting and governance reporting in coordination with the processor, So that fraud volumes, loss trends, recoveries, aging, and key risk indicators are visible to management and governance stakeholders</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>As a</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> Fraud Specialist, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>I want</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> to prepare fraud loss reporting and governance reporting in coordination with the processor, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>So that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> fraud volumes, loss trends, recoveries, aging, and key risk indicators are visible to management and governance stakeholders</t>
+          </r>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -801,7 +1241,47 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Given that a reporting period has closed, When the Fraud Specialist prepares the fraud loss and governance report, Then the report shall include fraud volumes, loss trends, recoveries, aging, and key risk indicators, and shall be delivered to the relevant governance forum within the defined reporting cadence.</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Given that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> a reporting period has closed, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>When</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> the Fraud Specialist prepares the fraud loss and governance report, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Then</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> the report shall include fraud volumes, loss trends, recoveries, aging, and key risk indicators, and shall be delivered to the relevant governance forum within the defined reporting cadence.</t>
+          </r>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
@@ -828,7 +1308,47 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>As a Fraud Specialist, I want to analyze authentication failures on an ongoing basis, So that I can identify patterns, root causes, and potential fraud-rule tuning opportunities</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>As a</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> Fraud Specialist, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>I want</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> to analyze authentication failures on an ongoing basis, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>So that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> I can identify patterns, root causes, and potential fraud-rule tuning opportunities</t>
+          </r>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -838,7 +1358,47 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Given that authentication failure data is available on an ongoing basis, When the Fraud Specialist conducts the periodic failure analysis, Then patterns and root causes shall be identified and documented, and any recommended fraud-rule tuning shall be raised for review.</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Given that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> authentication failure data is available on an ongoing basis, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>When</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> the Fraud Specialist conducts the periodic failure analysis, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Then</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> patterns and root causes shall be identified and documented, and any recommended fraud-rule tuning shall be raised for review.</t>
+          </r>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
@@ -865,7 +1425,47 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>As a Fraud Specialist, I want to prepare fraudulent disputes for submission to Visa VROL, So that fraud disputes are processed through VROL within Visa's required timeframes</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>As a</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> Fraud Specialist, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>I want</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> to prepare fraudulent disputes for submission to Visa VROL, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>So that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> fraud disputes are processed through VROL within Visa's required timeframes</t>
+          </r>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -875,7 +1475,47 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Given that a cardholder dispute has been confirmed as fraud, When the Fraud Specialist prepares the dispute case for submission, Then the case shall be packaged with all required documentation and provided for submission to VROL within Visa's mandated timeframe.</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Given that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> a cardholder dispute has been confirmed as fraud, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>When</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> the Fraud Specialist prepares the dispute case for submission, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Then</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> the case shall be packaged with all required documentation and provided for submission to VROL within Visa's mandated timeframe.</t>
+          </r>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
@@ -894,7 +1534,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="150" customHeight="1">
+    <row r="13" ht="165" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
           <t>1.9</t>
@@ -902,7 +1542,47 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>As a Fraud Monitoring System, I want to support the deployment, creation, modification, and deactivation of business rules in the production environment, across varying rule lengths, variables, rule syntax, and logic complexities, So that Fraud Specialists can configure and maintain effective fraud detection logic without requiring a code deployment</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>As a</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> Fraud Monitoring System, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>I want</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> to support the deployment, creation, modification, and deactivation of business rules in the production environment, across varying rule lengths, variables, rule syntax, and logic complexities, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>So that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> Fraud Specialists can configure and maintain effective fraud detection logic without requiring a code deployment</t>
+          </r>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
@@ -912,7 +1592,47 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Given that a Fraud Specialist has defined a new or modified business rule, When the rule is deployed, created, modified, or deactivated in the production environment, Then the system shall apply the change without requiring a code deployment or application restart, regardless of the rule's length, variables, syntax, or logic complexity.</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Given that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> a Fraud Specialist has defined a new or modified business rule, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>When</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> the rule is deployed, created, modified, or deactivated in the production environment, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Then</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> the system shall apply the change without requiring a code deployment or application restart, regardless of the rule's length, variables, syntax, or logic complexity.</t>
+          </r>
         </is>
       </c>
       <c r="E13" s="11" t="inlineStr">
@@ -931,7 +1651,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="105" customHeight="1">
+    <row r="14" ht="120" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
           <t>1.10</t>
@@ -939,7 +1659,47 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>As a Fraud Monitoring System, I want to provide interactive dashboards displaying solution health, transaction volumes, and alert activity, So that Fraud Specialists can monitor the fraud program's operational status in real time</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>As a</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> Fraud Monitoring System, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>I want</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> to provide interactive dashboards displaying solution health, transaction volumes, and alert activity, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>So that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> Fraud Specialists can monitor the fraud program's operational status in real time</t>
+          </r>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
@@ -949,7 +1709,47 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Given that the fraud monitoring system is in production, When a Fraud Specialist accesses the dashboard, Then the dashboard shall display current solution health status, transaction volumes, and alert activity, filterable by date range and status.</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Given that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> the fraud monitoring system is in production, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>When</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> a Fraud Specialist accesses the dashboard, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Then</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> the dashboard shall display current solution health status, transaction volumes, and alert activity, filterable by date range and status.</t>
+          </r>
         </is>
       </c>
       <c r="E14" s="11" t="inlineStr">
@@ -976,7 +1776,47 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>As a Fraud Specialist, I want the fraud monitoring dashboards to be reliably available and performant, So that I can monitor solution health, volumes, and alerts without delay or downtime</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>As a</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> Fraud Specialist, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>I want</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> the fraud monitoring dashboards to be reliably available and performant, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>So that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> I can monitor solution health, volumes, and alerts without delay or downtime</t>
+          </r>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
@@ -986,7 +1826,47 @@
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Given that the fraud monitoring dashboard is in use, When dashboard data is refreshed, Then updated volumes, alerts, and health status shall be reflected within the defined refresh interval, and the dashboard shall be available in accordance with Beem's defined system availability SLA.</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Given that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> the fraud monitoring dashboard is in use, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>When</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> dashboard data is refreshed, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Then</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> updated volumes, alerts, and health status shall be reflected within the defined refresh interval, and the dashboard shall be available in accordance with Beem's defined system availability SLA.</t>
+          </r>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
@@ -1013,7 +1893,47 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>As a Fraud Monitoring System, I want to automatically generate alerts for held transactions and send them to downstream systems in real time, So that held transactions are actioned promptly by the appropriate team or system</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>As a</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> Fraud Monitoring System, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>I want</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> to automatically generate alerts for held transactions and send them to downstream systems in real time, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>So that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> held transactions are actioned promptly by the appropriate team or system</t>
+          </r>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -1023,7 +1943,47 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Given that a transaction is held by the fraud monitoring system, When the hold is applied, Then an alert shall be automatically generated and transmitted to the applicable downstream system(s) in real time.</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Given that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> a transaction is held by the fraud monitoring system, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>When</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> the hold is applied, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Then</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> an alert shall be automatically generated and transmitted to the applicable downstream system(s) in real time.</t>
+          </r>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
@@ -1050,7 +2010,47 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>As a Fraud Monitoring System, I want to allow Fraud Specialists to view, create, and customize analytics and performance reports, So that the team can track and monitor fraud program performance and trends</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>As a</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> Fraud Monitoring System, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>I want</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> to allow Fraud Specialists to view, create, and customize analytics and performance reports, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>So that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> the team can track and monitor fraud program performance and trends</t>
+          </r>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -1060,7 +2060,47 @@
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Given that a Fraud Specialist requires a report to track or monitor fraud program performance, When the Fraud Specialist creates or customizes an analytics or performance report within the fraud monitoring system, Then the report shall be generated and made available for view, export, and ongoing use.</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Given that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> a Fraud Specialist requires a report to track or monitor fraud program performance, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>When</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> the Fraud Specialist creates or customizes an analytics or performance report within the fraud monitoring system, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Then</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> the report shall be generated and made available for view, export, and ongoing use.</t>
+          </r>
         </is>
       </c>
       <c r="E17" s="11" t="inlineStr">
@@ -1165,7 +2205,47 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>As an AML Specialist, I want to monitor, investigate, and disposition AML alerts arising from Visa Debit activity, So that suspicious activity is identified and actioned in accordance with Beem's AML program</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>As an</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> AML Specialist, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>I want</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> to monitor, investigate, and disposition AML alerts arising from Visa Debit activity, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>So that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> suspicious activity is identified and actioned in accordance with Beem's AML program</t>
+          </r>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -1175,7 +2255,47 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Given that Visa Debit transaction activity is monitored by the AML monitoring system, When an alert is generated for potentially suspicious activity, Then the AML Specialist shall investigate and disposition the alert (e.g., cleared, escalated, STR filed) and document the outcome.</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Given that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> Visa Debit transaction activity is monitored by the AML monitoring system, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>When</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> an alert is generated for potentially suspicious activity, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Then</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> the AML Specialist shall investigate and disposition the alert (e.g., cleared, escalated, STR filed) and document the outcome.</t>
+          </r>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
@@ -1202,7 +2322,47 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>As an AML Specialist, I want to perform ongoing sanctions screening of Visa Debit cardholders, So that cardholders are screened against OFAC SDN and other applicable sanctions lists at onboarding and on an ongoing basis</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>As an</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> AML Specialist, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>I want</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> to perform ongoing sanctions screening of Visa Debit cardholders, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>So that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> cardholders are screened against OFAC SDN and other applicable sanctions lists at onboarding and on an ongoing basis</t>
+          </r>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -1212,7 +2372,47 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Given that a cardholder is onboarded or an ongoing sanctions screening cycle occurs, When the cardholder's details are screened against OFAC SDN and other applicable sanctions lists, Then any potential match shall be flagged for AML Specialist review and disposition prior to further account activity, where required.</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Given that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> a cardholder is onboarded or an ongoing sanctions screening cycle occurs, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>When</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> the cardholder's details are screened against OFAC SDN and other applicable sanctions lists, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Then</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> any potential match shall be flagged for AML Specialist review and disposition prior to further account activity, where required.</t>
+          </r>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -1231,7 +2431,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="135" customHeight="1">
+    <row r="7" ht="120" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>2.3</t>
@@ -1239,7 +2439,47 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>As an AML Specialist, I want to assess FINTRAC reporting obligations arising from Visa Debit activity, So that I can determine whether a transaction triggers an STR, EFT, or LCT report</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>As an</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> AML Specialist, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>I want</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> to assess FINTRAC reporting obligations arising from Visa Debit activity, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>So that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> I can determine whether a transaction triggers an STR, EFT, or LCT report</t>
+          </r>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -1249,7 +2489,47 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Given that Visa Debit transaction activity meets or is suspected to meet FINTRAC reporting criteria, When the AML Specialist assesses the transaction, Then the AML Specialist shall determine whether an STR, EFT, and/or LCT report is required and document the assessment.</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Given that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> Visa Debit transaction activity meets or is suspected to meet FINTRAC reporting criteria, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>When</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> the AML Specialist assesses the transaction, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Then</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> the AML Specialist shall determine whether an STR, EFT, and/or LCT report is required and document the assessment.</t>
+          </r>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
@@ -1268,7 +2548,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="120" customHeight="1">
+    <row r="8" ht="135" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>2.4</t>
@@ -1276,7 +2556,47 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>As an AML Specialist, I want to prepare and submit regulatory reports where required, So that Beem meets its FINTRAC and other applicable regulatory reporting obligations for Visa Debit activity</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>As an</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> AML Specialist, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>I want</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> to prepare and submit regulatory reports where required, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>So that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> Beem meets its FINTRAC and other applicable regulatory reporting obligations for Visa Debit activity</t>
+          </r>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -1286,7 +2606,47 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Given that a regulatory reporting obligation (e.g., STR, EFT, LCT) has been identified for Visa Debit activity, When the AML Specialist prepares the report, Then the report shall be submitted to FINTRAC within the applicable regulatory timeframe and retained per record-keeping requirements.</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Given that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> a regulatory reporting obligation (e.g., STR, EFT, LCT) has been identified for Visa Debit activity, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>When</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> the AML Specialist prepares the report, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Then</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> the report shall be submitted to FINTRAC within the applicable regulatory timeframe and retained per record-keeping requirements.</t>
+          </r>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
@@ -1313,7 +2673,47 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>As an AML Specialist, I want to prepare management reporting for Visa Debit AML monitoring, So that AML alert volumes, escalations, STR filings, and key risk indicators are visible to management and governance stakeholders</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>As an</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> AML Specialist, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>I want</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> to prepare management reporting for Visa Debit AML monitoring, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>So that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> AML alert volumes, escalations, STR filings, and key risk indicators are visible to management and governance stakeholders</t>
+          </r>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
@@ -1323,7 +2723,47 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Given that a reporting period has closed, When the AML Specialist prepares the AML management report, Then the report shall include alert volumes, escalations, STR filings, and key risk indicators, and shall be delivered to the relevant governance forum within the defined reporting cadence.</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Given that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> a reporting period has closed, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>When</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> the AML Specialist prepares the AML management report, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Then</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> the report shall include alert volumes, escalations, STR filings, and key risk indicators, and shall be delivered to the relevant governance forum within the defined reporting cadence.</t>
+          </r>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
@@ -1350,7 +2790,47 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>As an AML Specialist, I want to maintain and tune AML monitoring rules for Visa Debit activity, So that the monitoring program remains effective at detecting suspicious activity specific to Visa Debit transaction types</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>As an</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> AML Specialist, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>I want</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> to maintain and tune AML monitoring rules for Visa Debit activity, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>So that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> the monitoring program remains effective at detecting suspicious activity specific to Visa Debit transaction types</t>
+          </r>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -1360,7 +2840,47 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Given that Visa Debit AML monitoring rules are in production, When the AML Specialist conducts periodic rule review and tuning, Then rule changes shall be assessed, tested, and documented, and approved changes shall be implemented in the AML monitoring system.</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Given that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> Visa Debit AML monitoring rules are in production, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>When</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> the AML Specialist conducts periodic rule review and tuning, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Then</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> rule changes shall be assessed, tested, and documented, and approved changes shall be implemented in the AML monitoring system.</t>
+          </r>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
@@ -1387,7 +2907,47 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>As an AML Monitoring System, I want to support the deployment, creation, modification, and deactivation of business rules in the production environment, across varying rule lengths, variables, rule syntax, and logic complexities, So that AML Specialists can configure and maintain effective AML detection logic without requiring a code deployment</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>As an</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> AML Monitoring System, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>I want</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> to support the deployment, creation, modification, and deactivation of business rules in the production environment, across varying rule lengths, variables, rule syntax, and logic complexities, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>So that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> AML Specialists can configure and maintain effective AML detection logic without requiring a code deployment</t>
+          </r>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -1397,7 +2957,47 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Given that an AML Specialist has defined a new or modified business rule, When the rule is deployed, created, modified, or deactivated in the production environment, Then the system shall apply the change without requiring a code deployment or application restart, regardless of the rule's length, variables, syntax, or logic complexity.</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Given that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> an AML Specialist has defined a new or modified business rule, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>When</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> the rule is deployed, created, modified, or deactivated in the production environment, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Then</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> the system shall apply the change without requiring a code deployment or application restart, regardless of the rule's length, variables, syntax, or logic complexity.</t>
+          </r>
         </is>
       </c>
       <c r="E11" s="11" t="inlineStr">
@@ -1424,7 +3024,47 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>As an AML Monitoring System, I want to screen cardholders against the OFAC Specially Designated Nationals and Blocked Persons List (SDN List) and other applicable sanctions lists at onboarding/issuance and on an ongoing basis, So that true matches are actioned immediately to prevent sanctioned individuals from transacting</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>As an</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> AML Monitoring System, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>I want</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> to screen cardholders against the OFAC Specially Designated Nationals and Blocked Persons List (SDN List) and other applicable sanctions lists at onboarding/issuance and on an ongoing basis, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>So that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> true matches are actioned immediately to prevent sanctioned individuals from transacting</t>
+          </r>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -1434,7 +3074,47 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Given that a cardholder is onboarded, issued a Visa Debit card, or included in an ongoing sanctions screening cycle, When the cardholder is screened against the OFAC SDN List and other applicable sanctions lists, Then any true match shall result in the cardholder's access being disabled, Visa being notified, and remediation being reported.</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Given that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> a cardholder is onboarded, issued a Visa Debit card, or included in an ongoing sanctions screening cycle, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>When</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> the cardholder is screened against the OFAC SDN List and other applicable sanctions lists, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Then</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> any true match shall result in the cardholder's access being disabled, Visa being notified, and remediation being reported.</t>
+          </r>
         </is>
       </c>
       <c r="E12" s="11" t="inlineStr">
@@ -1461,7 +3141,47 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>As an AML Monitoring System, I want to receive Visa Debit card data via an export mechanism such as an API, with sensitive data masked, So that the AML monitoring solution can perform screening, transaction monitoring, and case management on Visa Debit activity</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>As an</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> AML Monitoring System, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>I want</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> to receive Visa Debit card data via an export mechanism such as an API, with sensitive data masked, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>So that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> the AML monitoring solution can perform screening, transaction monitoring, and case management on Visa Debit activity</t>
+          </r>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
@@ -1471,7 +3191,47 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Given that Visa Debit transaction or cardholder data needs to be made available to the AML monitoring system, When the data export mechanism (e.g., API) runs, Then the data shall be delivered to the AML monitoring system with sensitive data elements masked in accordance with data protection requirements.</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Given that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> Visa Debit transaction or cardholder data needs to be made available to the AML monitoring system, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>When</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> the data export mechanism (e.g., API) runs, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Then</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> the data shall be delivered to the AML monitoring system with sensitive data elements masked in accordance with data protection requirements.</t>
+          </r>
         </is>
       </c>
       <c r="E13" s="11" t="inlineStr">
@@ -1490,7 +3250,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="105" customHeight="1">
+    <row r="14" ht="120" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
           <t>2.10</t>
@@ -1498,7 +3258,47 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>As an AML Monitoring System, I want to provide interactive dashboards displaying solution health, alert volumes, and case status, So that AML Specialists can monitor the AML program's operational status in real time</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>As an</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> AML Monitoring System, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>I want</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> to provide interactive dashboards displaying solution health, alert volumes, and case status, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>So that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> AML Specialists can monitor the AML program's operational status in real time</t>
+          </r>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
@@ -1508,7 +3308,47 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Given that the AML monitoring system is in production, When an AML Specialist accesses the dashboard, Then the dashboard shall display current solution health status, alert volumes, and case status, filterable by date range and status.</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Given that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> the AML monitoring system is in production, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>When</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> an AML Specialist accesses the dashboard, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Then</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> the dashboard shall display current solution health status, alert volumes, and case status, filterable by date range and status.</t>
+          </r>
         </is>
       </c>
       <c r="E14" s="11" t="inlineStr">
@@ -1535,7 +3375,47 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>As an AML Specialist, I want the AML monitoring dashboards to be reliably available and performant, So that I can monitor solution health, volumes, and alerts without delay or downtime</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>As an</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> AML Specialist, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>I want</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> the AML monitoring dashboards to be reliably available and performant, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>So that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> I can monitor solution health, volumes, and alerts without delay or downtime</t>
+          </r>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
@@ -1545,7 +3425,47 @@
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Given that the AML monitoring dashboard is in use, When dashboard data is refreshed, Then updated volumes, alerts, and health status shall be reflected within the defined refresh interval, and the dashboard shall be available in accordance with Beem's defined system availability SLA.</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Given that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> the AML monitoring dashboard is in use, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>When</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> dashboard data is refreshed, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Then</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> updated volumes, alerts, and health status shall be reflected within the defined refresh interval, and the dashboard shall be available in accordance with Beem's defined system availability SLA.</t>
+          </r>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
@@ -1572,7 +3492,47 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>As an AML Monitoring System, I want to allow AML Specialists to view, create, and customize analytics and performance reports, So that the team can track and monitor AML program performance and trends</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>As an</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> AML Monitoring System, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>I want</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> to allow AML Specialists to view, create, and customize analytics and performance reports, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>So that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> the team can track and monitor AML program performance and trends</t>
+          </r>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -1582,7 +3542,47 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Given that an AML Specialist requires a report to track or monitor AML program performance, When the AML Specialist creates or customizes an analytics or performance report within the AML monitoring system, Then the report shall be generated and made available for view, export, and ongoing use.</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Given that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> an AML Specialist requires a report to track or monitor AML program performance, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>When</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> the AML Specialist creates or customizes an analytics or performance report within the AML monitoring system, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Then</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> the report shall be generated and made available for view, export, and ongoing use.</t>
+          </r>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
@@ -1687,7 +3687,47 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>As a Compliance Officer, I want to perform the compliance portion of initial due diligence on net new Third Party Agents (TPAs), So that new TPAs meet Visa's compliance requirements before being onboarded into the Visa Debit program</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>As a</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> Compliance Officer, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>I want</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> to perform the compliance portion of initial due diligence on net new Third Party Agents (TPAs), </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>So that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> new TPAs meet Visa's compliance requirements before being onboarded into the Visa Debit program</t>
+          </r>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -1697,7 +3737,47 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Given that a net new TPA is being onboarded to support the Visa Debit program, When Compliance performs the compliance due diligence review, Then the TPA's compliance-related documentation and controls shall be reviewed and a compliance due diligence determination shall be documented prior to the TPA being onboarded.</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Given that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> a net new TPA is being onboarded to support the Visa Debit program, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>When</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> Compliance performs the compliance due diligence review, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Then</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> the TPA's compliance-related documentation and controls shall be reviewed and a compliance due diligence determination shall be documented prior to the TPA being onboarded.</t>
+          </r>
         </is>
       </c>
       <c r="E5" s="11" t="inlineStr">
@@ -1716,7 +3796,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="150" customHeight="1">
+    <row r="6" ht="135" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>3.2</t>
@@ -1724,7 +3804,47 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>As a Compliance Officer, I want to prepare and provide TPA-related reporting to Visa and/or the BIN Sponsor, So that Beem meets Visa's TPA registration, notification, and quarterly reporting requirements</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>As a</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> Compliance Officer, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>I want</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> to prepare and provide TPA-related reporting to Visa and/or the BIN Sponsor, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>So that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> Beem meets Visa's TPA registration, notification, and quarterly reporting requirements</t>
+          </r>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -1734,7 +3854,47 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Given that a TPA is registered, a TPA contract change occurs, or Visa/the BIN Sponsor requests quarterly TPA reporting, When Compliance prepares the applicable TPA report or notification, Then the report/notification shall be submitted to Visa and/or the BIN Sponsor within the applicable timeframe (e.g., within 5 business days for contract changes).</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Given that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> a TPA is registered, a TPA contract change occurs, or Visa/the BIN Sponsor requests quarterly TPA reporting, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>When</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> Compliance prepares the applicable TPA report or notification, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Then</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> the report/notification shall be submitted to Visa and/or the BIN Sponsor within the applicable timeframe (e.g., within 5 business days for contract changes).</t>
+          </r>
         </is>
       </c>
       <c r="E6" s="11" t="inlineStr">
@@ -1753,7 +3913,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="120" customHeight="1">
+    <row r="7" ht="105" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>3.3</t>
@@ -1761,7 +3921,47 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>As a Compliance Officer, I want to advise on the compliance coverage of net new TPA agreements, So that new TPA contracts meet Visa's contractual requirements for TPAs</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>As a</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> Compliance Officer, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>I want</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> to advise on the compliance coverage of net new TPA agreements, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>So that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> new TPA contracts meet Visa's contractual requirements for TPAs</t>
+          </r>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -1771,7 +3971,47 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Given that a net new TPA agreement is being drafted or finalized, When Compliance reviews the agreement, Then Compliance shall confirm the agreement includes the Visa-required contractual provisions and shall document any gaps or required amendments prior to execution.</t>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Given that</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> a net new TPA agreement is being drafted or finalized, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>When</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> Compliance reviews the agreement, </t>
+          </r>
+          <r>
+            <t>
+   </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>Then</t>
+          </r>
+          <r>
+            <t xml:space="preserve"> Compliance shall confirm the agreement includes the Visa-required contractual provisions and shall document any gaps or required amendments prior to execution.</t>
+          </r>
         </is>
       </c>
       <c r="E7" s="11" t="inlineStr">

</xml_diff>